<commit_message>
Add automation script for Login - Module and updated the test cases for login
</commit_message>
<xml_diff>
--- a/Signup_Automation_Test_Cases.xlsx
+++ b/Signup_Automation_Test_Cases.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sys\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F5DA151-FFB2-4BAC-AE57-988DB4F0A749}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29DAF880-CE28-464A-BDBA-7DE4C50586A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Signup" sheetId="1" r:id="rId1"/>
+    <sheet name="Login" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Signup!$A$1:$I$21</definedName>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="163">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -371,13 +372,154 @@
   </si>
   <si>
     <t>Success confirmation should be displayed and user should be logged in/redirected to the expected account page</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_AUTO_001</t>
+  </si>
+  <si>
+    <t>Login</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_AUTO_002</t>
+  </si>
+  <si>
+    <t>Login with valid registered credentials</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_AUTO_003</t>
+  </si>
+  <si>
+    <t>Login with invalid email and valid password</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_AUTO_004</t>
+  </si>
+  <si>
+    <t>Login with valid email and invalid password</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_AUTO_005</t>
+  </si>
+  <si>
+    <t>Login with invalid email and invalid password</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_AUTO_006</t>
+  </si>
+  <si>
+    <t>Verify Email field is mandatory</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_AUTO_007</t>
+  </si>
+  <si>
+    <t>Verify Password field is mandatory</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_AUTO_008</t>
+  </si>
+  <si>
+    <t>Verify login with both fields blank</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_AUTO_009</t>
+  </si>
+  <si>
+    <t>Verify invalid email format validation</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_AUTO_010</t>
+  </si>
+  <si>
+    <t>Verify login after logout</t>
+  </si>
+  <si>
+    <t>Verify successful login displays logged-in user state</t>
+  </si>
+  <si>
+    <t>Enter registered email and valid password and click Login</t>
+  </si>
+  <si>
+    <t>Valid registered email and password</t>
+  </si>
+  <si>
+    <t>User should be logged in successfully and expected logged-in user state should be displayed</t>
+  </si>
+  <si>
+    <t>Enter an unregistered email and valid password and click Login</t>
+  </si>
+  <si>
+    <t>Invalid email + valid password</t>
+  </si>
+  <si>
+    <t>Appropriate login error message should be displayed and user should not be logged in</t>
+  </si>
+  <si>
+    <t>Enter registered email and incorrect password and click Login</t>
+  </si>
+  <si>
+    <t>Valid email + invalid password</t>
+  </si>
+  <si>
+    <t>Enter invalid email and invalid password and click Login</t>
+  </si>
+  <si>
+    <t>Invalid email + invalid password</t>
+  </si>
+  <si>
+    <t>Leave Email blank, enter valid password and click Login</t>
+  </si>
+  <si>
+    <t>Email: Blank; Valid password</t>
+  </si>
+  <si>
+    <t>Required-field validation should be displayed and login should not proceed</t>
+  </si>
+  <si>
+    <t>Enter valid email, leave Password blank and click Login</t>
+  </si>
+  <si>
+    <t>Valid email; Password: Blank</t>
+  </si>
+  <si>
+    <t>Leave Email and Password blank and click Login</t>
+  </si>
+  <si>
+    <t>Email: Blank; Password: Blank</t>
+  </si>
+  <si>
+    <t>Enter invalid email format and valid password and click Login</t>
+  </si>
+  <si>
+    <t>Email: invalid-email; Valid password</t>
+  </si>
+  <si>
+    <t>Invalid email validation should be displayed and login should not proceed</t>
+  </si>
+  <si>
+    <t>Enter a password in the Password field</t>
+  </si>
+  <si>
+    <t>Login successfully, click Logout, and login again using valid credentials</t>
+  </si>
+  <si>
+    <t>User should be able to log in successfully after logout</t>
+  </si>
+  <si>
+    <t>Login using valid credentials and verify the resulting page/account state</t>
+  </si>
+  <si>
+    <t>Success message or logged-in user state should be displayed and expected account options should be available</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_AUTO_011</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -389,6 +531,20 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -426,7 +582,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -436,6 +592,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -739,7 +898,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22" style="3" customWidth="1"/>
@@ -1363,9 +1522,515 @@
         <v>17</v>
       </c>
     </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A22" s="4"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="4"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A23" s="2"/>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A25" s="2"/>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A26" s="2"/>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A27" s="2"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A28" s="2"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A29" s="2"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A30" s="2"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A31" s="2"/>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
+      <c r="I31" s="2"/>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A32" s="2"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
+      <c r="I32" s="2"/>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A33" s="2"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+      <c r="I33" s="2"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I21" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <mergeCells count="1">
+    <mergeCell ref="A22:I22"/>
+  </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C9D6CF3-800C-4D03-8976-ABF3F997FA35}">
+  <dimension ref="A1:I12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22" style="3" customWidth="1"/>
+    <col min="2" max="2" width="20" style="3" customWidth="1"/>
+    <col min="3" max="3" width="42" style="3" customWidth="1"/>
+    <col min="4" max="4" width="65" style="3" customWidth="1"/>
+    <col min="5" max="5" width="38" style="3" customWidth="1"/>
+    <col min="6" max="6" width="65" style="3" customWidth="1"/>
+    <col min="7" max="7" width="14" style="3" customWidth="1"/>
+    <col min="8" max="8" width="18" style="3" customWidth="1"/>
+    <col min="9" max="9" width="16" style="3" customWidth="1"/>
+    <col min="10" max="16384" width="8.7265625" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>